<commit_message>
Update CID file pathways to check
</commit_message>
<xml_diff>
--- a/InputData/web-app/CID/Check Input Data.xlsx
+++ b/InputData/web-app/CID/Check Input Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\CID\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163C0356-9559-4EF1-91ED-80F67B681CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28006605-55E0-4D64-8C4F-186187CD1EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
   <si>
     <t>CID Check Input Data</t>
   </si>
@@ -110,9 +110,6 @@
     <t>elec/BDTPTUMCF/BDTPTUMCF.csv</t>
   </si>
   <si>
-    <t>elec/RQSD/RQSD-BRQSD.csv</t>
-  </si>
-  <si>
     <t>elec/RQSD/RQSD-RQSD.csv</t>
   </si>
   <si>
@@ -186,6 +183,12 @@
   </si>
   <si>
     <t>trans/VTQaZ/VTQaZ-motorbikes.csv</t>
+  </si>
+  <si>
+    <t>elec/RQSD/RQSD-CQSD.csv</t>
+  </si>
+  <si>
+    <t>ctrl-settings/BEEEfEPS.csv</t>
   </si>
 </sst>
 </file>
@@ -572,18 +575,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB40378-4D92-6B46-95EC-BF41FEF6A51A}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.09765625" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="2"/>
+    <col min="1" max="1" width="15.06640625" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="10.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -591,14 +594,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -609,55 +612,55 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD815B91-4D8D-3140-B01A-98F4799EC5EA}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="1" max="1" width="20.265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -667,179 +670,178 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15C2FCA3-2250-8E45-A26E-181733CE1D14}">
-  <dimension ref="A1:A38"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A33"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="1" max="1" width="32.06640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -848,35 +850,35 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A5F9D-06D4-2548-AA03-82624CE63230}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="2" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct file path name for BEEEfEPS in the CID file
</commit_message>
<xml_diff>
--- a/InputData/web-app/CID/Check Input Data.xlsx
+++ b/InputData/web-app/CID/Check Input Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\CID\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28006605-55E0-4D64-8C4F-186187CD1EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53B9394-7029-461E-833C-0831EAA4BECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
   </bookViews>
@@ -188,7 +188,7 @@
     <t>elec/RQSD/RQSD-CQSD.csv</t>
   </si>
   <si>
-    <t>ctrl-settings/BEEEfEPS.csv</t>
+    <t>ctrl-settings/BEEEfEPS/BEEEfEPS.csv</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Add historical vintage subrange to avoid input data errors carrying through to the amount of start year electricity capacity
</commit_message>
<xml_diff>
--- a/InputData/web-app/CID/Check Input Data.xlsx
+++ b/InputData/web-app/CID/Check Input Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\CID\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53B9394-7029-461E-833C-0831EAA4BECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A25DF5-7E10-4531-832E-DD8163CD652B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
   <si>
     <t>CID Check Input Data</t>
   </si>
@@ -189,6 +189,9 @@
   </si>
   <si>
     <t>ctrl-settings/BEEEfEPS/BEEEfEPS.csv</t>
+  </si>
+  <si>
+    <t>ctrl-settings/MV/MV-historical</t>
   </si>
 </sst>
 </file>
@@ -849,7 +852,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A5F9D-06D4-2548-AA03-82624CE63230}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.3984375" style="1" bestFit="1" customWidth="1"/>
@@ -863,21 +866,26 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct file path name in CID file
</commit_message>
<xml_diff>
--- a/InputData/web-app/CID/Check Input Data.xlsx
+++ b/InputData/web-app/CID/Check Input Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\CID\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A25DF5-7E10-4531-832E-DD8163CD652B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91ABAFF7-5B2C-477F-9DEF-847C8320557E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
   </bookViews>
@@ -191,7 +191,7 @@
     <t>ctrl-settings/BEEEfEPS/BEEEfEPS.csv</t>
   </si>
   <si>
-    <t>ctrl-settings/MV/MV-historical</t>
+    <t>ctrl-settings/MV/MV-historical.csv</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
update CID file to remove IFStFS
</commit_message>
<xml_diff>
--- a/InputData/web-app/CID/Check Input Data.xlsx
+++ b/InputData/web-app/CID/Check Input Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\CID\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/todd/eps/eps-us/InputData/web-app/CID/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163C0356-9559-4EF1-91ED-80F67B681CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08472ACC-31FA-684C-B8E8-8DE1DA37EF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
+    <workbookView xWindow="28680" yWindow="620" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="48">
   <si>
     <t>CID Check Input Data</t>
   </si>
@@ -114,9 +114,6 @@
   </si>
   <si>
     <t>elec/RQSD/RQSD-RQSD.csv</t>
-  </si>
-  <si>
-    <t>indst/IFStFS/IFStFS.csv</t>
   </si>
   <si>
     <t>trans/BVTStL/BVTStL.csv</t>
@@ -572,18 +569,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB40378-4D92-6B46-95EC-BF41FEF6A51A}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.09765625" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="2"/>
+    <col min="1" max="1" width="15.140625" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="10.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -591,14 +588,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -609,55 +606,55 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD815B91-4D8D-3140-B01A-98F4799EC5EA}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="1" max="1" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -667,179 +664,168 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15C2FCA3-2250-8E45-A26E-181733CE1D14}">
-  <dimension ref="A1:A38"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="1" max="1" width="32.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -848,35 +834,35 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A5F9D-06D4-2548-AA03-82624CE63230}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.69921875" style="1"/>
+    <col min="1" max="1" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update CID check input data file list
</commit_message>
<xml_diff>
--- a/InputData/web-app/CID/Check Input Data.xlsx
+++ b/InputData/web-app/CID/Check Input Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\CID\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/todd/eps/eps-us/InputData/web-app/CID/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23430FE0-5759-4E08-B06F-388D855B8D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A3DEED-CDB4-EF4D-8CAD-6D26ADF52A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{20505A23-B03E-B349-AF36-73B0855D7AFA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
   <si>
     <t>CID Check Input Data</t>
   </si>
@@ -110,9 +110,6 @@
     <t>elec/BDTPTUMCF/BDTPTUMCF.csv</t>
   </si>
   <si>
-    <t>elec/RQSD/RQSD-RQSD.csv</t>
-  </si>
-  <si>
     <t>indst/IFStFS/IFStFS.csv</t>
   </si>
   <si>
@@ -179,13 +176,22 @@
     <t>trans/VTQaZ/VTQaZ-motorbikes.csv</t>
   </si>
   <si>
-    <t>elec/RQSD/RQSD-CQSD.csv</t>
-  </si>
-  <si>
     <t>ctrl-settings/BEEEfEPS/BEEEfEPS.csv</t>
   </si>
   <si>
     <t>ctrl-settings/MV/MV-historical.csv</t>
+  </si>
+  <si>
+    <t>elec/BEPQSD/BEPQSD-CQSD.csv</t>
+  </si>
+  <si>
+    <t>elec/BEPQSD/BEPQSD-RQSD.csv</t>
+  </si>
+  <si>
+    <t>elec/EPQSD/EPQSD-CQSD.csv</t>
+  </si>
+  <si>
+    <t>elec/EPQSD/EPQSD-RQSD.csv</t>
   </si>
 </sst>
 </file>
@@ -572,18 +578,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB40378-4D92-6B46-95EC-BF41FEF6A51A}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.06640625" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="10.6640625" style="2"/>
+    <col min="1" max="1" width="15" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="10.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -591,14 +597,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -609,55 +615,55 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD815B91-4D8D-3140-B01A-98F4799EC5EA}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.6640625" style="1"/>
+    <col min="1" max="1" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -667,210 +673,221 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15C2FCA3-2250-8E45-A26E-181733CE1D14}">
-  <dimension ref="A1:A33"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.06640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.6640625" style="1"/>
+    <col min="1" max="1" width="32" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A5F9D-06D4-2548-AA03-82624CE63230}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="10.6640625" style="1"/>
+    <col min="1" max="1" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>